<commit_message>
Rebuild s1_q02-q10 answer workbooks with per-part highlights and legend; Q2 embed-only
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TNVxQFJXojPDm4Z5hNnmdq
</commit_message>
<xml_diff>
--- a/practice/answers/s1_q03.xlsx
+++ b/practice/answers/s1_q03.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Answer" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Answer" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -22,7 +22,7 @@
     <numFmt numFmtId="166" formatCode="0.0"/>
     <numFmt numFmtId="167" formatCode="&quot;$&quot;#,##0.00"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -31,45 +31,10 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <name val="Arial"/>
       <b val="1"/>
-      <color rgb="004A7C59"/>
-      <sz val="13"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <color rgb="005C6B62"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <color rgb="0024302A"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Consolas"/>
-      <color rgb="002F5D46"/>
-      <sz val="9"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <b val="1"/>
-      <color rgb="0024302A"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <color rgb="005C6B62"/>
-      <sz val="9"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -78,12 +43,32 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="004A7C59"/>
+        <fgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F6EFD9"/>
+        <fgColor rgb="00D9EAD3"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F4CCCC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00CFE2F3"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9D2E9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FCE5CD"/>
       </patternFill>
     </fill>
   </fills>
@@ -99,44 +84,31 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="1" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="1" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="4" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="6" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="6" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="4" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="167" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -502,267 +474,341 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F18"/>
+  <dimension ref="A1:H25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="8" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="30" customWidth="1" min="6" max="6"/>
+    <col width="9" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="11" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
-    <row r="1" ht="18" customHeight="1">
+    <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Entering a delivery log</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="32" customHeight="1">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>The table was typed in from the question. Dates are real dates (right aligned), tonnes show one decimal, and the Charge column shows where the brackets have to go.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="18" customHeight="1"/>
-    <row r="4" ht="18" customHeight="1">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="B4" s="4" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Crop</t>
         </is>
       </c>
-      <c r="C4" s="4" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Tonnes</t>
         </is>
       </c>
-      <c r="D4" s="4" t="inlineStr">
-        <is>
-          <t>Km</t>
-        </is>
-      </c>
-      <c r="E4" s="4" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Km hauled</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>Days since previous</t>
+        </is>
+      </c>
+      <c r="F1" s="3" t="inlineStr">
         <is>
           <t>Charge</t>
         </is>
       </c>
-      <c r="F4" s="4" t="inlineStr">
-        <is>
-          <t>The formula in E</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="18" customHeight="1">
-      <c r="A5" s="5" t="n">
+    </row>
+    <row r="2">
+      <c r="A2" s="4" t="n">
         <v>46279</v>
       </c>
-      <c r="B5" s="6" t="inlineStr">
+      <c r="B2" t="inlineStr">
         <is>
           <t>Canola</t>
         </is>
       </c>
-      <c r="C5" s="7" t="n">
+      <c r="C2" s="5" t="n">
         <v>42.5</v>
       </c>
-      <c r="D5" s="8" t="n">
+      <c r="D2" t="n">
         <v>38</v>
       </c>
-      <c r="E5" s="9">
-        <f>(4.1+0.085*D5)*C5*(1-0.015)</f>
-        <v/>
-      </c>
-      <c r="F5" s="10">
-        <f>_xlfn.FORMULATEXT(E5)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="6" ht="18" customHeight="1">
-      <c r="A6" s="5" t="n">
+      <c r="E2" s="6" t="n"/>
+      <c r="F2" s="7">
+        <f>(4.10+0.085*D2)*C2*(1-0.015)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="n">
         <v>46283</v>
       </c>
-      <c r="B6" s="6" t="inlineStr">
+      <c r="B3" t="inlineStr">
         <is>
           <t>Canola</t>
         </is>
       </c>
-      <c r="C6" s="7" t="n">
+      <c r="C3" s="5" t="n">
         <v>38</v>
       </c>
-      <c r="D6" s="8" t="n">
+      <c r="D3" t="n">
         <v>52</v>
       </c>
-      <c r="E6" s="9">
-        <f>(4.1+0.085*D6)*C6*(1-0.015)</f>
-        <v/>
-      </c>
-      <c r="F6" s="10">
-        <f>_xlfn.FORMULATEXT(E6)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="7" ht="18" customHeight="1">
-      <c r="A7" s="5" t="n">
+      <c r="E3" s="8">
+        <f>A3-A2</f>
+        <v/>
+      </c>
+      <c r="F3" s="7">
+        <f>(4.10+0.085*D3)*C3*(1-0.015)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="n">
         <v>46288</v>
       </c>
-      <c r="B7" s="6" t="inlineStr">
+      <c r="B4" t="inlineStr">
         <is>
           <t>Wheat</t>
         </is>
       </c>
-      <c r="C7" s="7" t="n">
+      <c r="C4" s="5" t="n">
         <v>61.2</v>
       </c>
-      <c r="D7" s="8" t="n">
+      <c r="D4" t="n">
         <v>27</v>
       </c>
-      <c r="E7" s="9">
-        <f>(4.1+0.085*D7)*C7*(1-0.015)</f>
-        <v/>
-      </c>
-      <c r="F7" s="10">
-        <f>_xlfn.FORMULATEXT(E7)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="8" ht="18" customHeight="1">
-      <c r="A8" s="5" t="n">
+      <c r="E4" s="8">
+        <f>A4-A3</f>
+        <v/>
+      </c>
+      <c r="F4" s="7">
+        <f>(4.10+0.085*D4)*C4*(1-0.015)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="n">
         <v>46297</v>
       </c>
-      <c r="B8" s="6" t="inlineStr">
+      <c r="B5" t="inlineStr">
         <is>
           <t>Wheat</t>
         </is>
       </c>
-      <c r="C8" s="7" t="n">
+      <c r="C5" s="5" t="n">
         <v>55.8</v>
       </c>
-      <c r="D8" s="8" t="n">
+      <c r="D5" t="n">
         <v>64</v>
       </c>
-      <c r="E8" s="9">
-        <f>(4.1+0.085*D8)*C8*(1-0.015)</f>
-        <v/>
-      </c>
-      <c r="F8" s="10">
-        <f>_xlfn.FORMULATEXT(E8)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="9" ht="18" customHeight="1">
-      <c r="A9" s="5" t="n">
+      <c r="E5" s="8">
+        <f>A5-A4</f>
+        <v/>
+      </c>
+      <c r="F5" s="7">
+        <f>(4.10+0.085*D5)*C5*(1-0.015)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="n">
         <v>46304</v>
       </c>
-      <c r="B9" s="6" t="inlineStr">
+      <c r="B6" t="inlineStr">
         <is>
           <t>Barley</t>
         </is>
       </c>
-      <c r="C9" s="7" t="n">
+      <c r="C6" s="5" t="n">
         <v>47.3</v>
       </c>
-      <c r="D9" s="8" t="n">
+      <c r="D6" t="n">
         <v>41</v>
       </c>
-      <c r="E9" s="9">
-        <f>(4.1+0.085*D9)*C9*(1-0.015)</f>
-        <v/>
-      </c>
-      <c r="F9" s="10">
-        <f>_xlfn.FORMULATEXT(E9)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="10" ht="18" customHeight="1">
-      <c r="A10" s="11" t="inlineStr">
-        <is>
-          <t>Total</t>
-        </is>
-      </c>
-      <c r="C10" s="12">
-        <f>SUM(C5:C9)</f>
-        <v/>
-      </c>
-      <c r="E10" s="13">
-        <f>SUM(E5:E9)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="11" ht="18" customHeight="1"/>
-    <row r="12" ht="18" customHeight="1">
-      <c r="A12" s="11" t="inlineStr">
-        <is>
-          <t>COUNT of Tonnes (numbers)</t>
-        </is>
-      </c>
-      <c r="C12" s="14">
-        <f>COUNT(C5:C9)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="13" ht="18" customHeight="1">
-      <c r="A13" s="11" t="inlineStr">
-        <is>
-          <t>COUNTA of Crop (any entry)</t>
-        </is>
-      </c>
-      <c r="C13" s="14">
-        <f>COUNTA(B5:B9)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="14" ht="18" customHeight="1">
-      <c r="A14" s="11" t="inlineStr">
-        <is>
-          <t>COUNT of Crop (numbers only)</t>
-        </is>
-      </c>
-      <c r="C14" s="14">
-        <f>COUNT(B5:B9)</f>
-        <v/>
-      </c>
-      <c r="D14" s="15" t="inlineStr">
-        <is>
-          <t>zero -- the column holds text</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="18" customHeight="1"/>
-    <row r="16" ht="18" customHeight="1">
-      <c r="A16" s="11" t="inlineStr">
-        <is>
-          <t>The wrong formula</t>
-        </is>
-      </c>
-      <c r="E16" s="16">
-        <f>4.1+0.085*D5*C5*(1-0.015)</f>
-        <v/>
-      </c>
-      <c r="F16" s="10">
-        <f>_xlfn.FORMULATEXT(E16)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="17" ht="18" customHeight="1"/>
-    <row r="18" ht="30" customHeight="1">
-      <c r="A18" s="15" t="inlineStr">
-        <is>
-          <t>Without the brackets Excel multiplies before it adds, so the $4.10 base is charged once for the whole load instead of on every tonne. The base and the per-kilometre rate have to be grouped before either touches the tonnes.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="18" customHeight="1"/>
+      <c r="E6" s="8">
+        <f>A6-A5</f>
+        <v/>
+      </c>
+      <c r="F6" s="7">
+        <f>(4.10+0.085*D6)*C6*(1-0.015)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="F7" s="7">
+        <f>SUM(F2:F6)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="9" t="inlineStr">
+        <is>
+          <t>First to last (days)</t>
+        </is>
+      </c>
+      <c r="B8" s="10">
+        <f>A6-A2</f>
+        <v/>
+      </c>
+      <c r="D8" s="11" t="inlineStr">
+        <is>
+          <t>COUNT counts only numbers, and the Crop column holds text, so COUNT on it would return 0; COUNTA counts any non-empty cell.</t>
+        </is>
+      </c>
+      <c r="E8" s="9" t="n"/>
+      <c r="F8" s="9" t="n"/>
+      <c r="G8" s="9" t="n"/>
+      <c r="H8" s="9" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="9" t="inlineStr">
+        <is>
+          <t>COUNT of Tonnes</t>
+        </is>
+      </c>
+      <c r="B9" s="9">
+        <f>COUNT(C2:C6)</f>
+        <v/>
+      </c>
+      <c r="D9" s="9" t="n"/>
+      <c r="E9" s="9" t="n"/>
+      <c r="F9" s="9" t="n"/>
+      <c r="G9" s="9" t="n"/>
+      <c r="H9" s="9" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="9" t="inlineStr">
+        <is>
+          <t>COUNTA of Crop</t>
+        </is>
+      </c>
+      <c r="B10" s="9">
+        <f>COUNTA(B2:B6)</f>
+        <v/>
+      </c>
+      <c r="D10" s="9" t="n"/>
+      <c r="E10" s="9" t="n"/>
+      <c r="F10" s="9" t="n"/>
+      <c r="G10" s="9" t="n"/>
+      <c r="H10" s="9" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="12" t="inlineStr">
+        <is>
+          <t>That formula computes 4.10 + (0.085 x km x tonnes x 0.985): multiplication happens before addition, so the base rate is added once for the whole load instead of being charged on every tonne. The rates must be grouped first: =(4.10+0.085*D2)*C2*(1-0.015).</t>
+        </is>
+      </c>
+      <c r="B12" s="13" t="n"/>
+      <c r="C12" s="13" t="n"/>
+      <c r="D12" s="13" t="n"/>
+      <c r="E12" s="13" t="n"/>
+      <c r="F12" s="13" t="n"/>
+      <c r="G12" s="13" t="n"/>
+      <c r="H12" s="13" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="13" t="n"/>
+      <c r="B13" s="13" t="n"/>
+      <c r="C13" s="13" t="n"/>
+      <c r="D13" s="13" t="n"/>
+      <c r="E13" s="13" t="n"/>
+      <c r="F13" s="13" t="n"/>
+      <c r="G13" s="13" t="n"/>
+      <c r="H13" s="13" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="13" t="n"/>
+      <c r="B14" s="13" t="n"/>
+      <c r="C14" s="13" t="n"/>
+      <c r="D14" s="13" t="n"/>
+      <c r="E14" s="13" t="n"/>
+      <c r="F14" s="13" t="n"/>
+      <c r="G14" s="13" t="n"/>
+      <c r="H14" s="13" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="14" t="inlineStr">
+        <is>
+          <t>A date is stored as a number, which is what lets one be subtracted from another. Stored as text, date-shaped entries are converted inside a subtraction, but COUNT, SUM and AVERAGE skip text, so any range function over the column would silently return 0.</t>
+        </is>
+      </c>
+      <c r="B16" s="15" t="n"/>
+      <c r="C16" s="15" t="n"/>
+      <c r="D16" s="15" t="n"/>
+      <c r="E16" s="15" t="n"/>
+      <c r="F16" s="15" t="n"/>
+      <c r="G16" s="15" t="n"/>
+      <c r="H16" s="15" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="15" t="n"/>
+      <c r="B17" s="15" t="n"/>
+      <c r="C17" s="15" t="n"/>
+      <c r="D17" s="15" t="n"/>
+      <c r="E17" s="15" t="n"/>
+      <c r="F17" s="15" t="n"/>
+      <c r="G17" s="15" t="n"/>
+      <c r="H17" s="15" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="15" t="n"/>
+      <c r="B18" s="15" t="n"/>
+      <c r="C18" s="15" t="n"/>
+      <c r="D18" s="15" t="n"/>
+      <c r="E18" s="15" t="n"/>
+      <c r="F18" s="15" t="n"/>
+      <c r="G18" s="15" t="n"/>
+      <c r="H18" s="15" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="16" t="inlineStr">
+        <is>
+          <t>Part (a)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="6" t="inlineStr">
+        <is>
+          <t>Part (b)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="9" t="inlineStr">
+        <is>
+          <t>Part (c)</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="17" t="inlineStr">
+        <is>
+          <t>Part (d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="13" t="inlineStr">
+        <is>
+          <t>Part (e)</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="15" t="inlineStr">
+        <is>
+          <t>Part (f)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A18:F18"/>
+  <mergeCells count="3">
+    <mergeCell ref="D8:H10"/>
+    <mergeCell ref="A16:H18"/>
+    <mergeCell ref="A12:H14"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>